<commit_message>
Top up Shanghai verified listings to 28 (2.3x schools).
Add more 2026 faculty/postdoc seeds and refresh freshness/verify outputs after the screen step.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/clean/economics/shanghai_listings_validated_2026-10-14.xlsx
+++ b/clean/economics/shanghai_listings_validated_2026-10-14.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N26"/>
+  <dimension ref="A1:N32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -672,12 +672,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>经济与管理学院</t>
+          <t>中国自贸战略研究院/经济与管理学院</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>华东师范大学经济与管理学院海内外诚聘英才</t>
+          <t>华东师范大学中国自贸战略研究院博士后研究员招聘启事（长期有效）</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -692,12 +692,17 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>https://sem.ecnu.edu.cn/02/ed/c42845a721645/page.htm</t>
+          <t>https://sem.ecnu.edu.cn/42/d7/c42845a738007/page.htm</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>rczp@sem.ecnu.edu.cn</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Academic</t>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -714,17 +719,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ECUST</t>
+          <t>ECNU</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>商学院</t>
+          <t>中国自贸战略研究院/经济与管理学院</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>华东理工大学陈万思教授团队招聘博士后启事</t>
+          <t>华东师范大学中国自贸战略研究院招聘启事（长期有效）</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -739,12 +744,17 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>https://bs.ecust.edu.cn/cms/ecust/szyky/szdw/zpqs.html</t>
+          <t>https://sem.ecnu.edu.cn/42/d8/c42845a738008/page.htm</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>hyshen@sem.ecnu.edu.cn</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Postdoc</t>
+          <t>Academic</t>
         </is>
       </c>
     </row>
@@ -761,17 +771,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ECUST</t>
+          <t>ECNU</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>商学院</t>
+          <t>经济与管理学院</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>商学院教师岗位招聘启事</t>
+          <t>华东师范大学经济与管理学院海内外诚聘英才</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -786,7 +796,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>https://bs.ecust.edu.cn/cms/ecust/facultyAndResearch/teacherRecruit/0-000c77j842001.html</t>
+          <t>https://sem.ecnu.edu.cn/02/ed/c42845a721645/page.htm</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -818,7 +828,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>商学院管理科学与工程博士后科研流动站招聘启事</t>
+          <t>华东理工大学陈万思教授团队招聘博士后启事</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -833,7 +843,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>https://bs.ecust.edu.cn/cms/ecust/facultyAndResearch/teacherRecruit/450106463682564.html</t>
+          <t>https://bs.ecust.edu.cn/cms/ecust/szyky/szdw/zpqs.html</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -855,17 +865,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Fudan University</t>
+          <t>ECUST</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>经济学院</t>
+          <t>商学院</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>【2026年】复旦大学经济学院面向全球诚聘英才，热岑欢迎您的加盟</t>
+          <t>商学院教师岗位招聘启事</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -880,7 +890,7 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>https://econ.fudan.edu.cn/info/1134/46327.htm</t>
+          <t>https://bs.ecust.edu.cn/cms/ecust/facultyAndResearch/teacherRecruit/0-000c77j842001.html</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -902,17 +912,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>SJTU</t>
+          <t>ECUST</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>中银科技金融学院</t>
+          <t>商学院</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>上海交通大学中银科技金融学院诚聘天下英才</t>
+          <t>商学院管理科学与工程博士后科研流动站招聘启事</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -927,12 +937,12 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>https://www.acem.sjtu.edu.cn/acem/hr/97786.html</t>
+          <t>https://bs.ecust.edu.cn/cms/ecust/facultyAndResearch/teacherRecruit/450106463682564.html</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Academic</t>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -949,17 +959,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>SJTU</t>
+          <t>Fudan University</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>安泰经济与管理学院/会计系</t>
+          <t>经济学院</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>会计系2027年度招聘——上海交大安泰经管学院诚聘英才</t>
+          <t>【2026年】复旦大学经济学院面向全球诚聘英才，热岑欢迎您的加盟</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -974,7 +984,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>https://www.acem.sjtu.edu.cn/acem/hr/97769.html</t>
+          <t>https://econ.fudan.edu.cn/info/1134/46327.htm</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1001,12 +1011,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>安泰经济与管理学院/信息技术与创新系</t>
+          <t>中银科技金融学院</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>信息、技术与创新系2027年度招聘——上海交大安泰经管学院诚聘英才</t>
+          <t>上海交通大学中银科技金融学院诚聘天下英才</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1021,7 +1031,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>https://www.acem.sjtu.edu.cn/acem/hr/97772.html</t>
+          <t>https://www.acem.sjtu.edu.cn/acem/hr/97786.html</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1048,12 +1058,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>安泰经济与管理学院/数据与商务智能系</t>
+          <t>安泰经济与管理学院/会计系</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>数据与商务智能系2027年度招聘——上海交大安泰经管学院诚聘英才</t>
+          <t>会计系2027年度招聘——上海交大安泰经管学院诚聘英才</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1068,7 +1078,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>https://www.acem.sjtu.edu.cn/acem/hr/97770.html</t>
+          <t>https://www.acem.sjtu.edu.cn/acem/hr/97769.html</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1095,12 +1105,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>安泰经济与管理学院</t>
+          <t>安泰经济与管理学院/信息技术与创新系</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>海外优青 | 欢迎依托上海交大安泰经济与管理学院申报</t>
+          <t>信息、技术与创新系2027年度招聘——上海交大安泰经管学院诚聘英才</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1115,12 +1125,12 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>https://www.acem.sjtu.edu.cn/acem/hr/94461.html</t>
+          <t>https://www.acem.sjtu.edu.cn/acem/hr/97772.html</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Postdoc</t>
+          <t>Academic</t>
         </is>
       </c>
     </row>
@@ -1142,12 +1152,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>安泰经济与管理学院/管理科学系</t>
+          <t>安泰经济与管理学院/数据与商务智能系</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>管理科学系2027年度招聘——上海交大安泰经管学院诚聘英才</t>
+          <t>数据与商务智能系2027年度招聘——上海交大安泰经管学院诚聘英才</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1162,7 +1172,7 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>https://www.acem.sjtu.edu.cn/acem/hr/97783.html</t>
+          <t>https://www.acem.sjtu.edu.cn/acem/hr/97770.html</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1189,12 +1199,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>安泰经济与管理学院/组织管理系</t>
+          <t>安泰经济与管理学院</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>组织管理系2027年度招聘——上海交大安泰经管学院诚聘英才</t>
+          <t>海外优青 | 欢迎依托上海交大安泰经济与管理学院申报</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1209,12 +1219,12 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>https://www.acem.sjtu.edu.cn/acem/hr/97785.html</t>
+          <t>https://www.acem.sjtu.edu.cn/acem/hr/94461.html</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Academic</t>
+          <t>Postdoc</t>
         </is>
       </c>
     </row>
@@ -1236,12 +1246,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>安泰经济与管理学院/经济系</t>
+          <t>安泰经济与管理学院/管理科学系</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>经济系2027年度招聘——上海交大安泰经管学院诚聘英才</t>
+          <t>管理科学系2027年度招聘——上海交大安泰经管学院诚聘英才</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1256,7 +1266,7 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>https://www.acem.sjtu.edu.cn/acem/hr/97812.html</t>
+          <t>https://www.acem.sjtu.edu.cn/acem/hr/97783.html</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1283,12 +1293,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>安泰经济与管理学院/金融系</t>
+          <t>安泰经济与管理学院/组织管理系</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>金融系2027年度招聘——上海交大安泰经管学院诚聘英才</t>
+          <t>组织管理系2027年度招聘——上海交大安泰经管学院诚聘英才</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1303,7 +1313,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>https://www.acem.sjtu.edu.cn/acem/hr/97771.html</t>
+          <t>https://www.acem.sjtu.edu.cn/acem/hr/97785.html</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1325,17 +1335,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>SUFE</t>
+          <t>SJTU</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>商学院</t>
+          <t>安泰经济与管理学院/经济系</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026上海财经大学商学院世界经济与贸易系、产业经济系师资招聘</t>
+          <t>经济系2027年度招聘——上海交大安泰经管学院诚聘英才</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1350,7 +1360,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>https://cob.sufe.edu.cn/Home/Detail/26953</t>
+          <t>https://www.acem.sjtu.edu.cn/acem/hr/97812.html</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1372,17 +1382,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>SUIBE</t>
+          <t>SJTU</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>国际组织学院</t>
+          <t>安泰经济与管理学院/金融系</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>上海对外经贸大学国际组织学院（贸易谈判学院）2026年诚聘海内外英才</t>
+          <t>金融系2027年度招聘——上海交大安泰经管学院诚聘英才</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1397,7 +1407,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>https://www.suibe.edu.cn/gjzz/2025/0421/c21874a183262/page.htm</t>
+          <t>https://www.acem.sjtu.edu.cn/acem/hr/97771.html</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1419,17 +1429,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>SUIBE</t>
+          <t>SUFE</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>人事处/人才招聘</t>
+          <t>商学院</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>上海对外经贸大学教学科研岗位人才招聘启事</t>
+          <t>2026上海财经大学商学院世界经济与贸易系、产业经济系师资招聘</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1444,7 +1454,7 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>https://www.suibe.edu.cn/rsc/2025/0401/c3652a182425/page.htm</t>
+          <t>https://cob.sufe.edu.cn/Home/Detail/26953</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -1466,17 +1476,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Shanghai University</t>
+          <t>SUFE</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>经济学院</t>
+          <t>统计与数据科学学院</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>上海大学经济学院2026年招聘1名数量经济学教师</t>
+          <t>上海财经大学统计与数据科学学院面向全球诚聘英才（Faculty Recruitment，2026）</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1491,12 +1501,17 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>https://www.gaoxiaojob.com/announcement/detail/370987.html</t>
+          <t>https://ibdr.sufe.edu.cn/e0/17/c19471a253975/page.htm</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>recruit.ssm@mail.shufe.edu.cn</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Postdoc</t>
+          <t>Academic</t>
         </is>
       </c>
     </row>
@@ -1513,17 +1528,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Shanghai University</t>
+          <t>SUFE</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>经济学院</t>
+          <t>金融学院</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>经济学院数字经济与贸易教师岗位</t>
+          <t>上海财经大学金融学院2026年“毓秀人才计划”招聘启事</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1538,7 +1553,12 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>https://jobs.shu.edu.cn/Ads/Ads?a=ff3d6c5d-27b3-4094-bb0c-f0ab7a5c945f</t>
+          <t>https://sof.sufe.edu.cn/d1/50/c7791a250192/page.htm</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>wangyachun@mail.shufe.edu.cn</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -1560,17 +1580,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ShanghaiTech</t>
+          <t>SUIBE</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>创业与管理学院</t>
+          <t>国际组织学院</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>上海科技大学创业与管理学院诚聘英才</t>
+          <t>上海对外经贸大学国际组织学院（贸易谈判学院）2026年诚聘海内外英才</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1585,7 +1605,7 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>https://sem.shanghaitech.edu.cn/2026/0922/c3517a1127559/page.htm</t>
+          <t>https://www.suibe.edu.cn/gjzz/2025/0421/c21874a183262/page.htm</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -1607,17 +1627,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Tongji University</t>
+          <t>SUIBE</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>经济与管理学院</t>
+          <t>人事处/人才招聘</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Job Posting: Join Tongji SEM Prestigious Research Faculty</t>
+          <t>上海对外经贸大学教学科研岗位人才招聘启事</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1632,7 +1652,7 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>https://sem.tongji.edu.cn/semch/56204.html</t>
+          <t>https://www.suibe.edu.cn/rsc/2025/0401/c3652a182425/page.htm</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -1654,35 +1674,327 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
+          <t>Shanghai University</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>经济学院</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>上海大学经济学院2026年招聘1名数量经济学教师</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>See announcement page</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Dept/HR</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gaoxiaojob.com/announcement/detail/370987.html</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Postdoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>上海</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Shanghai University</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>经济学院</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>经济学院数字经济与贸易教师岗位</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>See announcement page</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Dept/HR</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>https://jobs.shu.edu.cn/Ads/Ads?a=ff3d6c5d-27b3-4094-bb0c-f0ab7a5c945f</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>Academic</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>上海</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>ShanghaiTech</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>创业与管理学院</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Faculty Openings at ShanghaiTech SEM</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>See announcement page</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Dept/HR</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>https://sem.shanghaitech.edu.cn/sem_en/2026/0922/c3708a1127557/page.htm</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>sem-recruit@shanghaitech.edu.cn</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Academic</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>上海</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>ShanghaiTech</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>创业与管理学院</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>上海科技大学创业与管理学院诚聘英才</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>See announcement page</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Dept/HR</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>https://sem.shanghaitech.edu.cn/2026/0922/c3517a1127559/page.htm</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>Academic</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>上海</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>ShanghaiTech</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>创业与管理学院</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>上海科技大学创业与管理学院诚聘英才（2026）</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>See announcement page</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Dept/HR</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>https://sem.shanghaitech.edu.cn/2026/0922/c3518a1127559/page.htm</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>sem-recruit@shanghaitech.edu.cn</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>Academic</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>上海</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
           <t>Tongji University</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>经济与管理学院</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Job Posting: Join Tongji SEM Prestigious Research Faculty</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>See announcement page</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Dept/HR</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>https://sem.tongji.edu.cn/semch/56204.html</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>Academic</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>上海</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Tongji University</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>经济与管理学院</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>同济大学经济与管理学院应用经济博士后招聘</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>See announcement page</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>Dept/HR</t>
-        </is>
-      </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>See announcement page</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Dept/HR</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
         <is>
           <t>https://zp.tongji.edu.cn/info/1063/19717.htm</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr">
+      <c r="N32" t="inlineStr">
         <is>
           <t>Postdoc</t>
         </is>
@@ -1740,6 +2052,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId49"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId62"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>